<commit_message>
Freyja singlar + album & record cards
</commit_message>
<xml_diff>
--- a/assets/Weekly stats.xlsx
+++ b/assets/Weekly stats.xlsx
@@ -1,24 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\hemsida\assets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C261DEF-80A9-4044-94E3-990A02CC039C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="10245" yWindow="2355" windowWidth="39660" windowHeight="17460" activeTab="1" xr2:uid="{BC7DF37A-909E-4C59-8EB4-84C90EA9873F}"/>
+    <workbookView xWindow="10245" yWindow="2355" windowWidth="29040" windowHeight="16440"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Chart1" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="125725"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -66,8 +60,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,18 +162,8 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="sv-SE"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -211,7 +195,7 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
+      <c:layout/>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -219,34 +203,12 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="2000" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mj-lt"/>
-              <a:ea typeface="+mj-ea"/>
-              <a:cs typeface="+mj-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="sv-SE"/>
-        </a:p>
-      </c:txPr>
     </c:title>
-    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -270,12 +232,11 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
               <c:f>Sheet1!$A$3:$A$55</c:f>
               <c:numCache>
-                <c:formatCode>d\-mmm\-yy</c:formatCode>
+                <c:formatCode>dd/mmm/yy</c:formatCode>
                 <c:ptCount val="53"/>
                 <c:pt idx="0">
                   <c:v>45950</c:v>
@@ -587,12 +548,12 @@
                   <c:v>94</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>93</c:v>
+                  <c:v>190</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-05AF-449E-9397-14DE8D09584C}"/>
             </c:ext>
@@ -621,12 +582,11 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
               <c:f>Sheet1!$A$3:$A$55</c:f>
               <c:numCache>
-                <c:formatCode>d\-mmm\-yy</c:formatCode>
+                <c:formatCode>dd/mmm/yy</c:formatCode>
                 <c:ptCount val="53"/>
                 <c:pt idx="0">
                   <c:v>45950</c:v>
@@ -908,12 +868,12 @@
                   <c:v>107</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>125</c:v>
+                  <c:v>137</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-05AF-449E-9397-14DE8D09584C}"/>
             </c:ext>
@@ -942,12 +902,11 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
               <c:f>Sheet1!$A$3:$A$55</c:f>
               <c:numCache>
-                <c:formatCode>d\-mmm\-yy</c:formatCode>
+                <c:formatCode>dd/mmm/yy</c:formatCode>
                 <c:ptCount val="53"/>
                 <c:pt idx="0">
                   <c:v>45950</c:v>
@@ -1153,7 +1112,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-05AF-449E-9397-14DE8D09584C}"/>
             </c:ext>
@@ -1179,12 +1138,11 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
               <c:f>Sheet1!$A$3:$A$55</c:f>
               <c:numCache>
-                <c:formatCode>d\-mmm\-yy</c:formatCode>
+                <c:formatCode>dd/mmm/yy</c:formatCode>
                 <c:ptCount val="53"/>
                 <c:pt idx="0">
                   <c:v>45950</c:v>
@@ -1357,28 +1315,20 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-05AF-449E-9397-14DE8D09584C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
+        <c:dLbls/>
         <c:gapWidth val="50"/>
         <c:overlap val="30"/>
-        <c:axId val="346696608"/>
-        <c:axId val="1828806191"/>
+        <c:axId val="161100160"/>
+        <c:axId val="161102080"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="4"/>
           <c:order val="4"/>
@@ -1409,7 +1359,7 @@
             <c:numRef>
               <c:f>Sheet1!$A$3:$A$55</c:f>
               <c:numCache>
-                <c:formatCode>d\-mmm\-yy</c:formatCode>
+                <c:formatCode>dd/mmm/yy</c:formatCode>
                 <c:ptCount val="53"/>
                 <c:pt idx="0">
                   <c:v>45950</c:v>
@@ -1721,7 +1671,7 @@
                   <c:v>201</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>219</c:v>
+                  <c:v>328</c:v>
                 </c:pt>
                 <c:pt idx="48">
                   <c:v>0</c:v>
@@ -1741,8 +1691,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-05AF-449E-9397-14DE8D09584C}"/>
             </c:ext>
@@ -1775,7 +1724,7 @@
             <c:numRef>
               <c:f>Sheet1!$A$3:$A$55</c:f>
               <c:numCache>
-                <c:formatCode>d\-mmm\-yy</c:formatCode>
+                <c:formatCode>dd/mmm/yy</c:formatCode>
                 <c:ptCount val="53"/>
                 <c:pt idx="0">
                   <c:v>45950</c:v>
@@ -1948,29 +1897,19 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-05AF-449E-9397-14DE8D09584C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
+        <c:dLbls/>
         <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="346696608"/>
-        <c:axId val="1828806191"/>
+        <c:axId val="161100160"/>
+        <c:axId val="161102080"/>
       </c:lineChart>
       <c:lineChart>
         <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="6"/>
           <c:order val="6"/>
@@ -2003,7 +1942,7 @@
             <c:numRef>
               <c:f>Sheet1!$A$3:$A$55</c:f>
               <c:numCache>
-                <c:formatCode>d\-mmm\-yy</c:formatCode>
+                <c:formatCode>dd/mmm/yy</c:formatCode>
                 <c:ptCount val="53"/>
                 <c:pt idx="0">
                   <c:v>45950</c:v>
@@ -2315,55 +2254,45 @@
                   <c:v>16899</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>17118</c:v>
+                  <c:v>17227</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>17118</c:v>
+                  <c:v>17227</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>17118</c:v>
+                  <c:v>17227</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>17118</c:v>
+                  <c:v>17227</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>17118</c:v>
+                  <c:v>17227</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>17118</c:v>
+                  <c:v>17227</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-05AF-449E-9397-14DE8D09584C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
+        <c:dLbls/>
         <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="346489200"/>
-        <c:axId val="1828810031"/>
+        <c:axId val="161110272"/>
+        <c:axId val="161108352"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="346696608"/>
+        <c:axId val="161100160"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:title>
-          <c:overlay val="0"/>
+          <c:layout/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -2392,9 +2321,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="d\-mmm\-yy" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
+        <c:numFmt formatCode="dd/mmm/yy" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -2429,20 +2356,17 @@
             <a:endParaRPr lang="sv-SE"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1828806191"/>
+        <c:crossAx val="161102080"/>
         <c:crosses val="autoZero"/>
-        <c:auto val="0"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:tickLblSkip val="4"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1828806191"/>
+        <c:axId val="161102080"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
@@ -2498,7 +2422,7 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="0"/>
+          <c:layout/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -2506,30 +2430,9 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="sv-SE"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="#.##0;\-#.##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -2558,16 +2461,15 @@
             <a:endParaRPr lang="sv-SE"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346696608"/>
+        <c:crossAx val="161100160"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1828810031"/>
+        <c:axId val="161108352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
         <c:axPos val="r"/>
         <c:title>
           <c:tx>
@@ -2600,7 +2502,7 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="0"/>
+          <c:layout/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -2608,30 +2510,9 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="sv-SE"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -2660,22 +2541,20 @@
             <a:endParaRPr lang="sv-SE"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="346489200"/>
+        <c:crossAx val="161110272"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:dateAx>
-        <c:axId val="346489200"/>
+        <c:axId val="161110272"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="1"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="d\-mmm\-yy" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1828810031"/>
+        <c:numFmt formatCode="dd/mmm/yy" sourceLinked="1"/>
+        <c:tickLblPos val="none"/>
+        <c:crossAx val="161108352"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -2691,7 +2570,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
-      <c:overlay val="0"/>
+      <c:layout/>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -2722,8 +2601,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -3300,7 +3178,7 @@
 </file>
 
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{A4DB0D66-11BC-4848-A11E-804ADE663E62}">
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3317,7 +3195,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12C9E449-515E-EC96-4A41-488CB1B02292}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{12C9E449-515E-EC96-4A41-488CB1B02292}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3383,7 +3261,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -3435,7 +3313,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -3649,26 +3527,26 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF015758-F449-42B6-B775-2DE6FC2FEA66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="1" customFormat="1" ht="20.25" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="2" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="2" customFormat="1" ht="16.5" thickTop="1" thickBot="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3688,7 +3566,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8">
       <c r="A3" s="3">
         <v>45950</v>
       </c>
@@ -3704,7 +3582,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8">
       <c r="A4" s="3">
         <f>A3+7</f>
         <v>45957</v>
@@ -3721,7 +3599,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8">
       <c r="A5" s="3">
         <f t="shared" ref="A5:A52" si="1">A4+7</f>
         <v>45964</v>
@@ -3738,7 +3616,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8">
       <c r="A6" s="3">
         <f t="shared" si="1"/>
         <v>45971</v>
@@ -3755,7 +3633,7 @@
         <v>1147</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="3">
         <f t="shared" si="1"/>
         <v>45978</v>
@@ -3772,7 +3650,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" s="3">
         <f t="shared" si="1"/>
         <v>45985</v>
@@ -3789,7 +3667,7 @@
         <v>1587</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" s="3">
         <f t="shared" si="1"/>
         <v>45992</v>
@@ -3806,7 +3684,7 @@
         <v>1808</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" s="3">
         <f t="shared" si="1"/>
         <v>45999</v>
@@ -3823,7 +3701,7 @@
         <v>2056</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="3">
         <f t="shared" si="1"/>
         <v>46006</v>
@@ -3840,7 +3718,7 @@
         <v>2284</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8">
       <c r="A12" s="3">
         <f t="shared" si="1"/>
         <v>46013</v>
@@ -3857,7 +3735,7 @@
         <v>2528</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8">
       <c r="A13" s="3">
         <f t="shared" si="1"/>
         <v>46020</v>
@@ -3877,7 +3755,7 @@
         <v>2853</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8">
       <c r="A14" s="3">
         <f t="shared" si="1"/>
         <v>46027</v>
@@ -3897,7 +3775,7 @@
         <v>3255</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8">
       <c r="A15" s="3">
         <f t="shared" si="1"/>
         <v>46034</v>
@@ -3917,7 +3795,7 @@
         <v>3494</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8">
       <c r="A16" s="3">
         <f t="shared" si="1"/>
         <v>46041</v>
@@ -3937,7 +3815,7 @@
         <v>3861</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8">
       <c r="A17" s="3">
         <f t="shared" si="1"/>
         <v>46048</v>
@@ -3957,7 +3835,7 @@
         <v>4275</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8">
       <c r="A18" s="3">
         <f t="shared" si="1"/>
         <v>46055</v>
@@ -3980,7 +3858,7 @@
         <v>4659</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8">
       <c r="A19" s="3">
         <f t="shared" si="1"/>
         <v>46062</v>
@@ -4000,7 +3878,7 @@
         <v>4999</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8">
       <c r="A20" s="3">
         <f t="shared" si="1"/>
         <v>46069</v>
@@ -4020,7 +3898,7 @@
         <v>5488</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8">
       <c r="A21" s="3">
         <f t="shared" si="1"/>
         <v>46076</v>
@@ -4043,7 +3921,7 @@
         <v>5918</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8">
       <c r="A22" s="3">
         <f t="shared" si="1"/>
         <v>46083</v>
@@ -4063,7 +3941,7 @@
         <v>6411</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8">
       <c r="A23" s="3">
         <f t="shared" si="1"/>
         <v>46090</v>
@@ -4083,7 +3961,7 @@
         <v>6782</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8">
       <c r="A24" s="3">
         <f t="shared" si="1"/>
         <v>46097</v>
@@ -4103,7 +3981,7 @@
         <v>7114</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8">
       <c r="A25" s="3">
         <f t="shared" si="1"/>
         <v>46104</v>
@@ -4123,7 +4001,7 @@
         <v>7427</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8">
       <c r="A26" s="3">
         <f t="shared" si="1"/>
         <v>46111</v>
@@ -4143,7 +4021,7 @@
         <v>7911</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8">
       <c r="A27" s="3">
         <f t="shared" si="1"/>
         <v>46118</v>
@@ -4163,7 +4041,7 @@
         <v>8351</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8">
       <c r="A28" s="3">
         <f t="shared" si="1"/>
         <v>46125</v>
@@ -4183,7 +4061,7 @@
         <v>8754</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8">
       <c r="A29" s="3">
         <f t="shared" si="1"/>
         <v>46132</v>
@@ -4203,7 +4081,7 @@
         <v>9183</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8">
       <c r="A30" s="3">
         <f t="shared" si="1"/>
         <v>46139</v>
@@ -4223,7 +4101,7 @@
         <v>9541</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8">
       <c r="A31" s="3">
         <f t="shared" si="1"/>
         <v>46146</v>
@@ -4243,7 +4121,7 @@
         <v>9847</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8">
       <c r="A32" s="3">
         <f t="shared" si="1"/>
         <v>46153</v>
@@ -4263,7 +4141,7 @@
         <v>10331</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8">
       <c r="A33" s="3">
         <f t="shared" si="1"/>
         <v>46160</v>
@@ -4286,7 +4164,7 @@
         <v>10893</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8">
       <c r="A34" s="3">
         <f t="shared" si="1"/>
         <v>46167</v>
@@ -4309,7 +4187,7 @@
         <v>11272</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8">
       <c r="A35" s="3">
         <f t="shared" si="1"/>
         <v>46174</v>
@@ -4332,7 +4210,7 @@
         <v>11582</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8">
       <c r="A36" s="3">
         <f t="shared" si="1"/>
         <v>46181</v>
@@ -4352,7 +4230,7 @@
         <v>11936</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8">
       <c r="A37" s="3">
         <f t="shared" si="1"/>
         <v>46188</v>
@@ -4372,7 +4250,7 @@
         <v>12264</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8">
       <c r="A38" s="3">
         <f t="shared" si="1"/>
         <v>46195</v>
@@ -4392,7 +4270,7 @@
         <v>12585</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8">
       <c r="A39" s="3">
         <f t="shared" si="1"/>
         <v>46202</v>
@@ -4412,7 +4290,7 @@
         <v>13017</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8">
       <c r="A40" s="3">
         <f t="shared" si="1"/>
         <v>46209</v>
@@ -4435,7 +4313,7 @@
         <v>13422</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8">
       <c r="A41" s="3">
         <f t="shared" si="1"/>
         <v>46216</v>
@@ -4455,7 +4333,7 @@
         <v>13919</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8">
       <c r="A42" s="3">
         <f t="shared" si="1"/>
         <v>46223</v>
@@ -4478,7 +4356,7 @@
         <v>14296</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8">
       <c r="A43" s="3">
         <f t="shared" si="1"/>
         <v>46230</v>
@@ -4498,7 +4376,7 @@
         <v>14738</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8">
       <c r="A44" s="3">
         <f t="shared" si="1"/>
         <v>46237</v>
@@ -4518,7 +4396,7 @@
         <v>15186</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8">
       <c r="A45" s="3">
         <f t="shared" si="1"/>
         <v>46244</v>
@@ -4538,7 +4416,7 @@
         <v>15851</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8">
       <c r="A46" s="3">
         <f t="shared" si="1"/>
         <v>46251</v>
@@ -4561,7 +4439,7 @@
         <v>16107</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8">
       <c r="A47" s="3">
         <f t="shared" si="1"/>
         <v>46258</v>
@@ -4584,7 +4462,7 @@
         <v>16391</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8">
       <c r="A48" s="3">
         <f t="shared" si="1"/>
         <v>46265</v>
@@ -4607,7 +4485,7 @@
         <v>16698</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8">
       <c r="A49" s="3">
         <f t="shared" si="1"/>
         <v>46272</v>
@@ -4627,30 +4505,30 @@
         <v>16899</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8">
       <c r="A50" s="3">
         <f t="shared" si="1"/>
         <v>46279</v>
       </c>
       <c r="B50">
-        <v>93</v>
+        <v>190</v>
       </c>
       <c r="C50">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="D50">
         <v>1</v>
       </c>
       <c r="F50">
         <f t="shared" si="0"/>
-        <v>219</v>
+        <v>328</v>
       </c>
       <c r="H50">
         <f t="shared" si="2"/>
-        <v>17118</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17227</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" s="3">
         <f t="shared" si="1"/>
         <v>46286</v>
@@ -4661,10 +4539,10 @@
       </c>
       <c r="H51">
         <f t="shared" si="2"/>
-        <v>17118</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17227</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" s="3">
         <f t="shared" si="1"/>
         <v>46293</v>
@@ -4675,10 +4553,10 @@
       </c>
       <c r="H52">
         <f t="shared" si="2"/>
-        <v>17118</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17227</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" s="3">
         <f t="shared" ref="A53:A55" si="3">A52+7</f>
         <v>46300</v>
@@ -4689,10 +4567,10 @@
       </c>
       <c r="H53">
         <f t="shared" ref="H53:H55" si="5">H52+F53</f>
-        <v>17118</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" s="5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>17227</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" s="5" customFormat="1" ht="15" thickBot="1">
       <c r="A54" s="4">
         <f t="shared" si="3"/>
         <v>46307</v>
@@ -4703,10 +4581,10 @@
       </c>
       <c r="H54" s="5">
         <f t="shared" si="5"/>
-        <v>17118</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+        <v>17227</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="15" thickTop="1">
       <c r="A55" s="3">
         <f t="shared" si="3"/>
         <v>46314</v>
@@ -4717,7 +4595,7 @@
       </c>
       <c r="H55">
         <f t="shared" si="5"/>
-        <v>17118</v>
+        <v>17227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>